<commit_message>
Add reviewed eleven-school rotation and independently sourced teaching facts
</commit_message>
<xml_diff>
--- a/site/exports/lzu-law.xlsx
+++ b/site/exports/lzu-law.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="Rd98f60fdc5664af0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="Rbafb522dee094b18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="R37e94107f40d4d8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R3ad7622bba184274"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="Ra324561ce9b646fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R53907357140f460f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="Rb73a28a1f6124bd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="R9a11358a99dd424a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R9a75166c71cd4235"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="R8bde8741dd8049c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T21_0" displayName="T21_0" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T39_0" displayName="T39_0" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="校区"/>
@@ -158,7 +158,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T21_1" displayName="T21_1" ref="A1:S12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T39_1" displayName="T39_1" ref="A1:S12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="事件类型"/>
@@ -185,7 +185,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T21_3" displayName="T21_3" ref="A1:L4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T39_3" displayName="T39_3" ref="A1:L4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="标题"/>
@@ -205,7 +205,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T21_4" displayName="T21_4" ref="A1:G7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T39_4" displayName="T39_4" ref="A1:G7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="来源ID"/>
@@ -420,7 +420,7 @@
     <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="55" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="110" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="26" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="26" hidden="0" customWidth="1"/>
@@ -528,7 +528,7 @@
         <x:v>兰州大学</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="64" customHeight="1">
+    <x:row r="4" ht="150" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>拜荣静</x:v>
       </x:c>
@@ -548,7 +548,7 @@
         <x:v>未见明确本人导师，不从主编、合作或个人指导学生身份反推。；精选论文非全集，仅官网列示书目链接，未逐篇出版者验证。；无本人学历陈述，不因博士生导师头衔推断学历。</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>分批核实资料，不是完整名录</x:v>
+        <x:v>分批核实资料，不是完整名录；部分职业履历，学历与师承仍有缺项；公开教学事实（非本人求学学历；教学／课程开设时间不是入学、授位或任职起点；不计入教育、任职、论文、导师统计及师承图）：刑事诉讼法；角色未披露；教学／课程开设时间：时间未披露；来源ID：bairongjing-source-2；https://laws.lzu.edu.cn/shiziduiwu/jiaoshou/2025/0610/312596.html</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str">
         <x:v>公开个人页（时效以核对日为准）</x:v>
@@ -564,7 +564,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c26d9d9a3e64764"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52551256995946d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1117,7 +1117,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R115cda7ec96d46f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcb5516134e944ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1350,7 +1350,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05d12e1da80b4b48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9703b59aa6e64cc0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1532,7 +1532,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fc7ff0d6fed41db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R291c30b0b6cf45f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>